<commit_message>
docs: tambah data mentah + mapping import PT Kode Niaga Tama (KNT)
File invoice asli KNT (rincian_faktur_penjualan_ptkodeniagatama...xlsx,
182rb baris) untuk referensi task020 (parser alias dinamis + rollback
per-import). Sekalian mapping classification rules + channel divisions
KNT yang sudah disiapkan (siap upload manual lewat halaman Import).

Repo private, sudah ada preseden sama untuk data MKO sebelumnya.
</commit_message>
<xml_diff>
--- a/docs-v2/template/template_import_channel_divisions_template.xlsx
+++ b/docs-v2/template/template_import_channel_divisions_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\pacman\e-dashbord\docs-v2\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B20AE344-4711-4532-B0C2-FA31F99DE12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F4F795-485D-4B1E-A544-F70BB8B97BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="2580" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1920" windowWidth="23040" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Channel Divisions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
   <si>
     <t>Template Import Channel Divisions</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>SALES SUPPORT JKT</t>
+  </si>
+  <si>
+    <t>SDR WEST CARD</t>
   </si>
 </sst>
 </file>
@@ -506,8 +509,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.796875" customWidth="1"/>
     <col min="2" max="2" width="48.796875" customWidth="1"/>
@@ -537,7 +540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -545,7 +548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -553,7 +556,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -561,7 +564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -569,7 +572,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -577,7 +580,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -585,7 +588,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -593,7 +596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -601,7 +604,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -609,7 +612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -727,6 +730,14 @@
       </c>
       <c r="B27" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>